<commit_message>
fix: traduz valores de status e resultado para portugues
</commit_message>
<xml_diff>
--- a/data/processed/tabela_partidas_tratada.xlsx
+++ b/data/processed/tabela_partidas_tratada.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -530,7 +530,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -575,7 +575,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -628,7 +628,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -636,7 +636,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -734,7 +734,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -742,7 +742,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -787,7 +787,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -795,7 +795,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -848,7 +848,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -893,7 +893,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J17" t="n">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J19" t="n">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J20" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J21" t="n">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J22" t="n">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J23" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J24" t="n">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J25" t="n">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J27" t="n">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J29" t="n">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J30" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J31" t="n">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>POSTPONED</t>
+          <t>ADIADO</t>
         </is>
       </c>
       <c r="J32" t="n">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J33" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J34" t="n">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J35" t="n">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L35" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J36" t="n">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L37" t="n">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J38" t="n">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L38" t="n">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L39" t="n">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J41" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L41" t="n">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J42" t="n">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L42" t="n">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J43" t="n">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L43" t="n">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J44" t="n">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L44" t="n">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J45" t="n">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J46" t="n">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L46" t="n">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L47" t="n">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L48" t="n">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L49" t="n">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J50" t="n">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L50" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L51" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J52" t="n">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J53" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L53" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L54" t="n">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L55" t="n">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J56" t="n">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L56" t="n">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J57" t="n">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L57" t="n">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J58" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L58" t="n">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J59" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L59" t="n">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L60" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J61" t="n">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L61" t="n">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J62" t="n">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L63" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J64" t="n">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L64" t="n">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J65" t="n">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L65" t="n">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J66" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L66" t="n">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J67" t="n">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L67" t="n">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J68" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L68" t="n">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J69" t="n">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L69" t="n">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L70" t="n">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L71" t="n">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J72" t="n">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L72" t="n">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J73" t="n">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L73" t="n">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J74" t="n">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L74" t="n">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J75" t="n">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L75" t="n">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J76" t="n">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L76" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J77" t="n">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L77" t="n">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J78" t="n">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L78" t="n">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J79" t="n">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L79" t="n">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J80" t="n">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L80" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J81" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L81" t="n">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J82" t="n">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L82" t="n">
@@ -4801,7 +4801,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J83" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J84" t="n">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J85" t="n">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L85" t="n">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J86" t="n">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J87" t="n">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J88" t="n">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L88" t="n">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J89" t="n">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J90" t="n">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L90" t="n">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J91" t="n">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L91" t="n">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J92" t="n">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L92" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J93" t="n">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L93" t="n">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J94" t="n">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L94" t="n">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J95" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L95" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J96" t="n">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L96" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J97" t="n">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L97" t="n">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J98" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L98" t="n">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J99" t="n">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L99" t="n">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J100" t="n">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L100" t="n">
@@ -5755,7 +5755,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J101" t="n">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L101" t="n">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J102" t="n">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L102" t="n">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J103" t="n">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L103" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J104" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L104" t="n">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J105" t="n">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L105" t="n">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J106" t="n">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L106" t="n">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J107" t="n">
@@ -6081,7 +6081,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L107" t="n">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J108" t="n">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L109" t="n">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L110" t="n">
@@ -6285,7 +6285,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J111" t="n">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -6338,7 +6338,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J112" t="n">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L112" t="n">
@@ -6391,7 +6391,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J113" t="n">
@@ -6399,7 +6399,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -6444,7 +6444,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J114" t="n">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L114" t="n">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J115" t="n">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J116" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J117" t="n">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J118" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J119" t="n">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J120" t="n">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J121" t="n">
@@ -6823,7 +6823,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J122" t="n">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J123" t="n">
@@ -6929,7 +6929,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -6974,7 +6974,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J124" t="n">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J125" t="n">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J126" t="n">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J127" t="n">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J128" t="n">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J129" t="n">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J130" t="n">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J131" t="n">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J132" t="n">
@@ -7406,7 +7406,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J133" t="n">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J134" t="n">
@@ -7512,7 +7512,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J135" t="n">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J136" t="n">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J137" t="n">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J138" t="n">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -7769,7 +7769,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J139" t="n">
@@ -7777,7 +7777,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L139" t="n">
@@ -7822,7 +7822,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J140" t="n">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J141" t="n">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J142" t="n">
@@ -7936,7 +7936,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J143" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J144" t="n">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J145" t="n">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J146" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J147" t="n">
@@ -8201,7 +8201,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J148" t="n">
@@ -8254,7 +8254,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L148" t="n">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J149" t="n">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -8350,7 +8350,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J150" t="n">
@@ -8358,7 +8358,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J151" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -8452,7 +8452,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J152" t="n">
@@ -8460,7 +8460,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J153" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J154" t="n">
@@ -8562,7 +8562,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -8605,7 +8605,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J155" t="n">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J156" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J157" t="n">
@@ -8715,7 +8715,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J158" t="n">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J159" t="n">
@@ -8817,7 +8817,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J160" t="n">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J161" t="n">
@@ -8919,7 +8919,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -8962,7 +8962,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J162" t="n">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -9013,7 +9013,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J163" t="n">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J164" t="n">
@@ -9072,7 +9072,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J165" t="n">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J166" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -9217,7 +9217,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J167" t="n">
@@ -9225,7 +9225,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -9268,7 +9268,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J168" t="n">
@@ -9276,7 +9276,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J169" t="n">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -9370,7 +9370,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J170" t="n">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J171" t="n">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L171" t="n">
@@ -9472,7 +9472,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J172" t="n">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -9523,7 +9523,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J173" t="n">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -9574,7 +9574,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J174" t="n">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -9625,7 +9625,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J175" t="n">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -9676,7 +9676,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J176" t="n">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L176" t="n">
@@ -9727,7 +9727,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J177" t="n">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>AWAY_TEAM</t>
+          <t>VISITANTE</t>
         </is>
       </c>
       <c r="L177" t="n">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J178" t="n">
@@ -9786,7 +9786,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="J179" t="n">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>HOME_TEAM</t>
+          <t>MANDANTE</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J242" t="n">
@@ -12337,7 +12337,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J243" t="n">
@@ -12376,7 +12376,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J244" t="n">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J245" t="n">
@@ -12454,7 +12454,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J246" t="n">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J247" t="n">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J248" t="n">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J249" t="n">
@@ -12610,7 +12610,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J250" t="n">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J251" t="n">
@@ -12688,7 +12688,7 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J252" t="n">
@@ -12727,7 +12727,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J253" t="n">
@@ -12766,7 +12766,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J254" t="n">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J255" t="n">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J256" t="n">
@@ -12883,7 +12883,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J257" t="n">
@@ -12922,7 +12922,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J258" t="n">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J259" t="n">
@@ -13000,7 +13000,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J260" t="n">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J261" t="n">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J262" t="n">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J263" t="n">
@@ -13156,7 +13156,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J264" t="n">
@@ -13195,7 +13195,7 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J265" t="n">
@@ -13234,7 +13234,7 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J266" t="n">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J267" t="n">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J268" t="n">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J269" t="n">
@@ -13390,7 +13390,7 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J270" t="n">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J271" t="n">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J272" t="n">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J273" t="n">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J274" t="n">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J275" t="n">
@@ -13624,7 +13624,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J276" t="n">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J277" t="n">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J278" t="n">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J279" t="n">
@@ -13780,7 +13780,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J280" t="n">
@@ -13819,7 +13819,7 @@
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J281" t="n">
@@ -13858,7 +13858,7 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J282" t="n">
@@ -13897,7 +13897,7 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J283" t="n">
@@ -13936,7 +13936,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J284" t="n">
@@ -13975,7 +13975,7 @@
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J285" t="n">
@@ -14014,7 +14014,7 @@
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J286" t="n">
@@ -14053,7 +14053,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J287" t="n">
@@ -14092,7 +14092,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J288" t="n">
@@ -14131,7 +14131,7 @@
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J289" t="n">
@@ -14170,7 +14170,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J290" t="n">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J291" t="n">
@@ -14248,7 +14248,7 @@
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J292" t="n">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J293" t="n">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J294" t="n">
@@ -14365,7 +14365,7 @@
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J295" t="n">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J296" t="n">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J297" t="n">
@@ -14482,7 +14482,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J298" t="n">
@@ -14521,7 +14521,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J299" t="n">
@@ -14560,7 +14560,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J300" t="n">
@@ -14599,7 +14599,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J301" t="n">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J302" t="n">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J303" t="n">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J304" t="n">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J305" t="n">
@@ -14794,7 +14794,7 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J306" t="n">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J307" t="n">
@@ -14872,7 +14872,7 @@
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J308" t="n">
@@ -14911,7 +14911,7 @@
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J309" t="n">
@@ -14950,7 +14950,7 @@
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J310" t="n">
@@ -14989,7 +14989,7 @@
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J311" t="n">
@@ -15028,7 +15028,7 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J312" t="n">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J313" t="n">
@@ -15106,7 +15106,7 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J314" t="n">
@@ -15145,7 +15145,7 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J315" t="n">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J316" t="n">
@@ -15223,7 +15223,7 @@
       </c>
       <c r="I317" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J317" t="n">
@@ -15262,7 +15262,7 @@
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J318" t="n">
@@ -15301,7 +15301,7 @@
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J319" t="n">
@@ -15340,7 +15340,7 @@
       </c>
       <c r="I320" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J320" t="n">
@@ -15379,7 +15379,7 @@
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J321" t="n">
@@ -15418,7 +15418,7 @@
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J322" t="n">
@@ -15457,7 +15457,7 @@
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J323" t="n">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="I324" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J324" t="n">
@@ -15535,7 +15535,7 @@
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J325" t="n">
@@ -15574,7 +15574,7 @@
       </c>
       <c r="I326" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J326" t="n">
@@ -15613,7 +15613,7 @@
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J327" t="n">
@@ -15652,7 +15652,7 @@
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J328" t="n">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J329" t="n">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J330" t="n">
@@ -15769,7 +15769,7 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J331" t="n">
@@ -15808,7 +15808,7 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J332" t="n">
@@ -15847,7 +15847,7 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J333" t="n">
@@ -15886,7 +15886,7 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J334" t="n">
@@ -15925,7 +15925,7 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J335" t="n">
@@ -15964,7 +15964,7 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J336" t="n">
@@ -16003,7 +16003,7 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J337" t="n">
@@ -16042,7 +16042,7 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J338" t="n">
@@ -16081,7 +16081,7 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J339" t="n">
@@ -16120,7 +16120,7 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J340" t="n">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J341" t="n">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J342" t="n">
@@ -16237,7 +16237,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J343" t="n">
@@ -16276,7 +16276,7 @@
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J344" t="n">
@@ -16315,7 +16315,7 @@
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J345" t="n">
@@ -16354,7 +16354,7 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J346" t="n">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J347" t="n">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J348" t="n">
@@ -16471,7 +16471,7 @@
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J349" t="n">
@@ -16510,7 +16510,7 @@
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J350" t="n">
@@ -16549,7 +16549,7 @@
       </c>
       <c r="I351" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J351" t="n">
@@ -16588,7 +16588,7 @@
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J352" t="n">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J353" t="n">
@@ -16666,7 +16666,7 @@
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J354" t="n">
@@ -16705,7 +16705,7 @@
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J355" t="n">
@@ -16744,7 +16744,7 @@
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J356" t="n">
@@ -16783,7 +16783,7 @@
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J357" t="n">
@@ -16822,7 +16822,7 @@
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J358" t="n">
@@ -16861,7 +16861,7 @@
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J359" t="n">
@@ -16900,7 +16900,7 @@
       </c>
       <c r="I360" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J360" t="n">
@@ -16939,7 +16939,7 @@
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J361" t="n">
@@ -16978,7 +16978,7 @@
       </c>
       <c r="I362" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J362" t="n">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J363" t="n">
@@ -17056,7 +17056,7 @@
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J364" t="n">
@@ -17095,7 +17095,7 @@
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J365" t="n">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J366" t="n">
@@ -17173,7 +17173,7 @@
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J367" t="n">
@@ -17212,7 +17212,7 @@
       </c>
       <c r="I368" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J368" t="n">
@@ -17251,7 +17251,7 @@
       </c>
       <c r="I369" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J369" t="n">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I370" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J370" t="n">
@@ -17329,7 +17329,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J371" t="n">
@@ -17368,7 +17368,7 @@
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J372" t="n">
@@ -17407,7 +17407,7 @@
       </c>
       <c r="I373" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J373" t="n">
@@ -17446,7 +17446,7 @@
       </c>
       <c r="I374" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J374" t="n">
@@ -17485,7 +17485,7 @@
       </c>
       <c r="I375" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J375" t="n">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="I376" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J376" t="n">
@@ -17563,7 +17563,7 @@
       </c>
       <c r="I377" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J377" t="n">
@@ -17602,7 +17602,7 @@
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J378" t="n">
@@ -17641,7 +17641,7 @@
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J379" t="n">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J380" t="n">
@@ -17719,7 +17719,7 @@
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>SCHEDULED</t>
+          <t>AGENDADO</t>
         </is>
       </c>
       <c r="J381" t="n">

</xml_diff>